<commit_message>
Certificacion 100% - Corregidos nulos en CONDICION DEUDA y DIAS VENCIDOS
</commit_message>
<xml_diff>
--- a/data/clean/datos_limpios.xlsx
+++ b/data/clean/datos_limpios.xlsx
@@ -560,10 +560,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -622,10 +620,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -684,10 +680,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -746,10 +740,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -808,10 +800,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -870,10 +860,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -932,10 +920,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -994,10 +980,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1056,10 +1040,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1118,10 +1100,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1180,10 +1160,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1242,10 +1220,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1304,10 +1280,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1366,10 +1340,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1428,10 +1400,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N16" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1492,10 +1462,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N17" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1554,10 +1522,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N18" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1618,10 +1584,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N19" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1676,10 +1640,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N20" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1734,10 +1696,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1792,10 +1752,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N22" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1850,10 +1808,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N23" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1914,10 +1870,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N24" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1978,10 +1932,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N25" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -2040,10 +1992,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -2102,10 +2052,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N27" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2164,10 +2112,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N28" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2226,10 +2172,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N29" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -2288,10 +2232,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N30" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2350,10 +2292,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N31" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2412,10 +2352,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N32" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2474,10 +2412,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N33" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2536,10 +2472,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N34" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -2598,10 +2532,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N35" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -2660,10 +2592,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N36" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -2722,10 +2652,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N37" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -2784,10 +2712,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N38" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2846,10 +2772,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -2908,10 +2832,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N40" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -2970,10 +2892,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N41" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -3032,10 +2952,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N42" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -3094,10 +3012,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N43" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -3156,10 +3072,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N44" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -3220,10 +3134,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N45" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -3278,10 +3190,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N46" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -3336,10 +3246,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N47" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -3394,10 +3302,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N48" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -3452,10 +3358,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -3516,10 +3420,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N50" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -3580,10 +3482,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N51" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -3642,10 +3542,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N52" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -3704,10 +3602,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N53" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -3766,10 +3662,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N54" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -3828,10 +3722,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N55" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -3890,10 +3782,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N56" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -3952,10 +3842,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N57" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -4014,10 +3902,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N58" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -4076,10 +3962,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N59" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -4138,10 +4022,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N60" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -4200,10 +4082,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N61" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -4262,10 +4142,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N62" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -4324,10 +4202,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N63" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -4386,10 +4262,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N64" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -4448,10 +4322,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N65" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -4510,10 +4382,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N66" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -4572,10 +4442,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N67" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -4634,10 +4502,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N68" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -4696,10 +4562,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N69" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -4758,10 +4622,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N70" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -4822,10 +4684,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N71" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -4880,10 +4740,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N72" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -4938,10 +4796,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N73" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -4996,10 +4852,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N74" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -5054,10 +4908,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N75" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -5118,10 +4970,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N76" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -5182,10 +5032,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N77" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -5244,10 +5092,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N78" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -5306,10 +5152,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N79" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N79" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -5368,10 +5212,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N80" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -5430,10 +5272,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N81" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N81" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -5492,10 +5332,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N82" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -5554,10 +5392,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N83" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -5616,10 +5452,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N84" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -5678,10 +5512,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N85" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -5740,10 +5572,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N86" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N86" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -5802,10 +5632,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N87" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N87" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -5864,10 +5692,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N88" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N88" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -5926,10 +5752,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N89" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N89" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -5988,10 +5812,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N90" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N90" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -6050,10 +5872,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N91" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -6112,10 +5932,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N92" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N92" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -6174,10 +5992,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N93" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N93" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -6236,10 +6052,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N94" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N94" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -6298,10 +6112,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N95" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N95" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -6360,10 +6172,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N96" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N96" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -6424,10 +6234,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N97" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N97" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -6482,10 +6290,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N98" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N98" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -6540,10 +6346,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N99" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N99" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -6598,10 +6402,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N100" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N100" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -6656,10 +6458,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N101" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N101" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -6720,10 +6520,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N102" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N102" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -6784,10 +6582,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N103" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N103" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -6846,10 +6642,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N104" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N104" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -6908,10 +6702,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N105" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N105" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -6970,10 +6762,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N106" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N106" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -7032,10 +6822,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N107" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N107" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -7094,10 +6882,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N108" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N108" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -7156,10 +6942,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N109" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N109" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -7218,10 +7002,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N110" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N110" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -7280,10 +7062,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N111" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N111" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -7342,10 +7122,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N112" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N112" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -7404,10 +7182,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N113" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N113" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -7466,10 +7242,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N114" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N114" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -7528,10 +7302,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N115" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N115" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -7590,10 +7362,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N116" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N116" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="117">
@@ -7652,10 +7422,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N117" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N117" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="118">
@@ -7714,10 +7482,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N118" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N118" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="119">
@@ -7776,10 +7542,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N119" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N119" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -7838,10 +7602,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N120" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N120" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="121">
@@ -7900,10 +7662,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N121" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N121" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -7962,10 +7722,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N122" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N122" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -8026,10 +7784,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N123" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N123" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="124">
@@ -8084,10 +7840,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N124" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N124" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="125">
@@ -8142,10 +7896,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N125" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N125" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="126">
@@ -8200,10 +7952,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N126" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N126" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -8258,10 +8008,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N127" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N127" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -8322,10 +8070,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N128" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N128" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -8386,10 +8132,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N129" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N129" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="130">
@@ -8448,10 +8192,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N130" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N130" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="131">
@@ -8510,10 +8252,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N131" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N131" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -8572,10 +8312,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N132" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N132" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="133">
@@ -8634,10 +8372,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N133" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N133" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -8696,10 +8432,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N134" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N134" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -8758,10 +8492,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N135" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N135" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="136">
@@ -8820,10 +8552,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N136" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N136" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -8882,10 +8612,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N137" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N137" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="138">
@@ -8944,10 +8672,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N138" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N138" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -9006,10 +8732,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N139" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N139" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="140">
@@ -9068,10 +8792,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N140" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N140" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="141">
@@ -9130,10 +8852,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N141" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N141" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -9192,10 +8912,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N142" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N142" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="143">
@@ -9254,10 +8972,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N143" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N143" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="144">
@@ -9316,10 +9032,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N144" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N144" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="145">
@@ -9378,10 +9092,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N145" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N145" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -9440,10 +9152,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N146" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N146" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -9502,10 +9212,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N147" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N147" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -9564,10 +9272,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N148" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N148" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -9628,10 +9334,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N149" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N149" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -9686,10 +9390,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N150" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N150" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="151">
@@ -9744,10 +9446,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N151" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N151" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="152">
@@ -9802,10 +9502,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N152" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N152" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="153">
@@ -9860,10 +9558,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N153" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N153" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="154">
@@ -9924,10 +9620,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N154" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N154" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -9988,10 +9682,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N155" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N155" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -10050,10 +9742,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N156" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N156" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="157">
@@ -10112,10 +9802,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N157" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N157" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="158">
@@ -10174,10 +9862,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N158" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N158" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="159">
@@ -10236,10 +9922,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N159" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N159" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="160">
@@ -10298,10 +9982,8 @@
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N160" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N160" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="161">
@@ -10320,9 +10002,11 @@
         </is>
       </c>
       <c r="E161" s="2" t="n">
-        <v>46100.6898490629</v>
-      </c>
-      <c r="F161" t="inlineStr"/>
+        <v>46100.6898490625</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
       <c r="G161" t="inlineStr">
         <is>
           <t>SOLES</t>
@@ -10344,16 +10028,18 @@
           <t>DEUDA BANCOS</t>
         </is>
       </c>
-      <c r="L161" t="inlineStr"/>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>PENDIENTE DE PAGO</t>
+        </is>
+      </c>
       <c r="M161" t="inlineStr">
         <is>
           <t>2026-03-19T16:33:22.964043</t>
         </is>
       </c>
-      <c r="N161" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N161" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Solo exportar columnas originales, DOLARES=0 para SOLES
</commit_message>
<xml_diff>
--- a/data/clean/datos_limpios.xlsx
+++ b/data/clean/datos_limpios.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N161"/>
+  <dimension ref="A1:L161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,16 +493,6 @@
           <t>CONDICION DEUDA</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>_limpieza_fecha</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>_limpieza_version</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -555,14 +545,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -615,14 +597,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -675,14 +649,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -735,14 +701,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -795,14 +753,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -855,14 +805,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -915,14 +857,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -975,14 +909,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1035,14 +961,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1095,14 +1013,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1155,14 +1065,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1215,14 +1117,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N13" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1275,14 +1169,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1335,14 +1221,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N15" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1378,7 +1256,7 @@
         <v>2998.38</v>
       </c>
       <c r="I16" t="n">
-        <v>869.095652173913</v>
+        <v>0</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1394,14 +1272,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N16" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1440,7 +1310,7 @@
         <v>4280.91</v>
       </c>
       <c r="I17" t="n">
-        <v>1240.843478260869</v>
+        <v>0</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1456,14 +1326,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N17" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1500,7 +1362,7 @@
         <v>519.91</v>
       </c>
       <c r="I18" t="n">
-        <v>150.6985507246377</v>
+        <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1516,14 +1378,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N18" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1578,14 +1432,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1618,7 +1464,7 @@
         <v>13000</v>
       </c>
       <c r="I20" t="n">
-        <v>3768.115942028986</v>
+        <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1634,14 +1480,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1674,7 +1512,7 @@
         <v>21000</v>
       </c>
       <c r="I21" t="n">
-        <v>6086.95652173913</v>
+        <v>0</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1690,14 +1528,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1730,7 +1560,7 @@
         <v>21000</v>
       </c>
       <c r="I22" t="n">
-        <v>6086.95652173913</v>
+        <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1746,14 +1576,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1786,7 +1608,7 @@
         <v>8000</v>
       </c>
       <c r="I23" t="n">
-        <v>2318.840579710145</v>
+        <v>0</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1802,14 +1624,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1848,7 +1662,7 @@
         <v>1950</v>
       </c>
       <c r="I24" t="n">
-        <v>565.2173913043478</v>
+        <v>0</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1864,14 +1678,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N24" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1926,14 +1732,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N25" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1970,7 +1768,7 @@
         <v>2625</v>
       </c>
       <c r="I26" t="n">
-        <v>760.8695652173913</v>
+        <v>0</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1986,14 +1784,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -2030,7 +1820,7 @@
         <v>4030</v>
       </c>
       <c r="I27" t="n">
-        <v>1168.115942028986</v>
+        <v>0</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2046,14 +1836,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N27" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2090,7 +1872,7 @@
         <v>3250</v>
       </c>
       <c r="I28" t="n">
-        <v>942.0289855072464</v>
+        <v>0</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2106,14 +1888,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N28" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2167,14 +1941,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N29" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2227,14 +1993,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N30" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2287,14 +2045,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N31" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2347,14 +2097,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N32" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2407,14 +2149,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N33" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2467,14 +2201,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N34" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2527,14 +2253,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N35" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2587,14 +2305,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N36" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2647,14 +2357,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N37" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2707,14 +2409,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N38" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2767,14 +2461,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N39" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2827,14 +2513,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N40" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2887,14 +2565,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N41" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2947,14 +2617,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N42" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2990,7 +2652,7 @@
         <v>9435.165555555561</v>
       </c>
       <c r="I43" t="n">
-        <v>2734.830595813206</v>
+        <v>0</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -3006,14 +2668,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N43" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -3050,7 +2704,7 @@
         <v>9668.43349206349</v>
       </c>
       <c r="I44" t="n">
-        <v>2802.444490453186</v>
+        <v>0</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -3066,14 +2720,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N44" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -3128,14 +2774,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N45" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -3168,7 +2806,7 @@
         <v>9901.70142857143</v>
       </c>
       <c r="I46" t="n">
-        <v>2870.058385093168</v>
+        <v>0</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -3184,14 +2822,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N46" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -3224,7 +2854,7 @@
         <v>10018.3353968254</v>
       </c>
       <c r="I47" t="n">
-        <v>2903.865332413159</v>
+        <v>0</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -3240,14 +2870,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N47" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -3280,7 +2902,7 @@
         <v>10134.9693650794</v>
       </c>
       <c r="I48" t="n">
-        <v>2937.672279733159</v>
+        <v>0</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -3296,14 +2918,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N48" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -3336,7 +2950,7 @@
         <v>10251.6033333333</v>
       </c>
       <c r="I49" t="n">
-        <v>2971.47922705313</v>
+        <v>0</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -3352,14 +2966,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N49" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -3398,7 +3004,7 @@
         <v>10368.2373015873</v>
       </c>
       <c r="I50" t="n">
-        <v>3005.28617437313</v>
+        <v>0</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -3414,14 +3020,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N50" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -3476,14 +3074,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N51" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -3520,7 +3110,7 @@
         <v>10601.5052380952</v>
       </c>
       <c r="I52" t="n">
-        <v>3072.900069013102</v>
+        <v>0</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3536,14 +3126,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N52" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -3580,7 +3162,7 @@
         <v>10718.1392063492</v>
       </c>
       <c r="I53" t="n">
-        <v>3106.707016333101</v>
+        <v>0</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3596,14 +3178,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N53" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -3640,7 +3214,7 @@
         <v>10834.7731746032</v>
       </c>
       <c r="I54" t="n">
-        <v>3140.513963653101</v>
+        <v>0</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3656,14 +3230,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N54" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -3717,14 +3283,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N55" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3777,14 +3335,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N56" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3837,14 +3387,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N57" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3897,14 +3439,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N58" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3957,14 +3491,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N59" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4017,14 +3543,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N60" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4077,14 +3595,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N61" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4137,14 +3647,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N62" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4197,14 +3699,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N63" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4257,14 +3751,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N64" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4317,14 +3803,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N65" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4377,14 +3855,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N66" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4437,14 +3907,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N67" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4497,14 +3959,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N68" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4540,7 +3994,7 @@
         <v>12584.2826984127</v>
       </c>
       <c r="I69" t="n">
-        <v>3647.618173452956</v>
+        <v>0</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
@@ -4556,14 +4010,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N69" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -4600,7 +4046,7 @@
         <v>12817.5506349206</v>
       </c>
       <c r="I70" t="n">
-        <v>3715.232068092927</v>
+        <v>0</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -4616,14 +4062,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N70" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -4678,14 +4116,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N71" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -4718,7 +4148,7 @@
         <v>13050.8185714286</v>
       </c>
       <c r="I72" t="n">
-        <v>3782.845962732927</v>
+        <v>0</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -4734,14 +4164,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N72" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -4774,7 +4196,7 @@
         <v>13167.4525396825</v>
       </c>
       <c r="I73" t="n">
-        <v>3816.652910052898</v>
+        <v>0</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -4790,14 +4212,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N73" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -4830,7 +4244,7 @@
         <v>13284.0865079365</v>
       </c>
       <c r="I74" t="n">
-        <v>3850.459857372898</v>
+        <v>0</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
@@ -4846,14 +4260,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N74" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -4886,7 +4292,7 @@
         <v>13400.7204761905</v>
       </c>
       <c r="I75" t="n">
-        <v>3884.266804692898</v>
+        <v>0</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -4902,14 +4308,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N75" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -4948,7 +4346,7 @@
         <v>13517.3544444444</v>
       </c>
       <c r="I76" t="n">
-        <v>3918.073752012869</v>
+        <v>0</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -4964,14 +4362,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M76" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N76" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -5026,14 +4416,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M77" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N77" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -5070,7 +4452,7 @@
         <v>13750.6223809524</v>
       </c>
       <c r="I78" t="n">
-        <v>3985.687646652869</v>
+        <v>0</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
@@ -5086,14 +4468,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N78" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -5130,7 +4504,7 @@
         <v>13867.2563492063</v>
       </c>
       <c r="I79" t="n">
-        <v>4019.49459397284</v>
+        <v>0</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -5146,14 +4520,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M79" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N79" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -5190,7 +4556,7 @@
         <v>13983.8903174603</v>
       </c>
       <c r="I80" t="n">
-        <v>4053.30154129284</v>
+        <v>0</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
@@ -5206,14 +4572,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N80" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -5267,14 +4625,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N81" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -5327,14 +4677,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N82" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -5387,14 +4729,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N83" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -5447,14 +4781,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N84" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -5507,14 +4833,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N85" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -5567,14 +4885,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N86" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -5627,14 +4937,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N87" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -5687,14 +4989,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N88" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -5747,14 +5041,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N89" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -5807,14 +5093,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N90" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -5867,14 +5145,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N91" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -5927,14 +5197,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M92" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N92" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -5987,14 +5249,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N93" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -6047,14 +5301,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N94" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -6090,7 +5336,7 @@
         <v>15733.3998412699</v>
       </c>
       <c r="I95" t="n">
-        <v>4560.405751092724</v>
+        <v>0</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -6106,14 +5352,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M95" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N95" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -6150,7 +5388,7 @@
         <v>15966.6677777778</v>
       </c>
       <c r="I96" t="n">
-        <v>4628.019645732696</v>
+        <v>0</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -6166,14 +5404,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M96" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N96" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -6228,14 +5458,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M97" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N97" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -6268,7 +5490,7 @@
         <v>16199.9357142858</v>
       </c>
       <c r="I98" t="n">
-        <v>4695.633540372695</v>
+        <v>0</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
@@ -6284,14 +5506,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M98" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N98" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -6324,7 +5538,7 @@
         <v>16316.5696825397</v>
       </c>
       <c r="I99" t="n">
-        <v>4729.440487692666</v>
+        <v>0</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
@@ -6340,14 +5554,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M99" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N99" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -6380,7 +5586,7 @@
         <v>16433.2036507937</v>
       </c>
       <c r="I100" t="n">
-        <v>4763.247435012667</v>
+        <v>0</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -6396,14 +5602,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M100" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N100" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -6436,7 +5634,7 @@
         <v>16549.8376190477</v>
       </c>
       <c r="I101" t="n">
-        <v>4797.054382332666</v>
+        <v>0</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
@@ -6452,14 +5650,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M101" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N101" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -6498,7 +5688,7 @@
         <v>16666.4715873016</v>
       </c>
       <c r="I102" t="n">
-        <v>4830.861329652637</v>
+        <v>0</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -6514,14 +5704,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M102" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N102" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -6576,14 +5758,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M103" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N103" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -6620,7 +5794,7 @@
         <v>16899.7395238096</v>
       </c>
       <c r="I104" t="n">
-        <v>4898.475224292637</v>
+        <v>0</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
@@ -6636,14 +5810,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M104" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N104" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -6680,7 +5846,7 @@
         <v>17016.3734920635</v>
       </c>
       <c r="I105" t="n">
-        <v>4932.282171612608</v>
+        <v>0</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
@@ -6696,14 +5862,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M105" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N105" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -6740,7 +5898,7 @@
         <v>17133.0074603175</v>
       </c>
       <c r="I106" t="n">
-        <v>4966.089118932609</v>
+        <v>0</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
@@ -6756,14 +5914,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M106" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N106" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -6817,14 +5967,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N107" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -6877,14 +6019,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N108" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -6937,14 +6071,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N109" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -6997,14 +6123,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N110" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -7057,14 +6175,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N111" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -7117,14 +6227,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M112" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N112" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -7177,14 +6279,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M113" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N113" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -7237,14 +6331,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M114" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N114" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -7297,14 +6383,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M115" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N115" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -7357,14 +6435,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N116" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -7417,14 +6487,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M117" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N117" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -7477,14 +6539,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N118" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -7537,14 +6591,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N119" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -7597,14 +6643,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M120" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N120" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -7640,7 +6678,7 @@
         <v>18882.516984127</v>
       </c>
       <c r="I121" t="n">
-        <v>5473.193328732464</v>
+        <v>0</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
@@ -7656,14 +6694,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M121" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N121" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -7700,7 +6730,7 @@
         <v>19115.784920635</v>
       </c>
       <c r="I122" t="n">
-        <v>5540.807223372463</v>
+        <v>0</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -7716,14 +6746,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M122" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N122" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -7778,14 +6800,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M123" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N123" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="124">
@@ -7818,7 +6832,7 @@
         <v>19349.0528571429</v>
       </c>
       <c r="I124" t="n">
-        <v>5608.421118012434</v>
+        <v>0</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
@@ -7834,14 +6848,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M124" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N124" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="125">
@@ -7874,7 +6880,7 @@
         <v>19465.6868253969</v>
       </c>
       <c r="I125" t="n">
-        <v>5642.228065332434</v>
+        <v>0</v>
       </c>
       <c r="J125" t="inlineStr">
         <is>
@@ -7890,14 +6896,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M125" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N125" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="126">
@@ -7930,7 +6928,7 @@
         <v>19582.3207936508</v>
       </c>
       <c r="I126" t="n">
-        <v>5676.035012652405</v>
+        <v>0</v>
       </c>
       <c r="J126" t="inlineStr">
         <is>
@@ -7946,14 +6944,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M126" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N126" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -7986,7 +6976,7 @@
         <v>19698.9547619048</v>
       </c>
       <c r="I127" t="n">
-        <v>5709.841959972405</v>
+        <v>0</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -8002,14 +6992,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M127" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N127" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -8048,7 +7030,7 @@
         <v>19815.5887301588</v>
       </c>
       <c r="I128" t="n">
-        <v>5743.648907292406</v>
+        <v>0</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -8064,14 +7046,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M128" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N128" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -8126,14 +7100,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M129" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N129" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="130">
@@ -8170,7 +7136,7 @@
         <v>20048.8566666667</v>
       </c>
       <c r="I130" t="n">
-        <v>5811.262801932377</v>
+        <v>0</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
@@ -8186,14 +7152,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M130" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N130" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="131">
@@ -8230,7 +7188,7 @@
         <v>20165.4906349207</v>
       </c>
       <c r="I131" t="n">
-        <v>5845.069749252377</v>
+        <v>0</v>
       </c>
       <c r="J131" t="inlineStr">
         <is>
@@ -8246,14 +7204,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M131" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N131" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -8290,7 +7240,7 @@
         <v>20282.1246031746</v>
       </c>
       <c r="I132" t="n">
-        <v>5878.876696572348</v>
+        <v>0</v>
       </c>
       <c r="J132" t="inlineStr">
         <is>
@@ -8306,14 +7256,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M132" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N132" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="133">
@@ -8367,14 +7309,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N133" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -8427,14 +7361,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N134" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -8487,14 +7413,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M135" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N135" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -8547,14 +7465,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M136" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N136" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -8607,14 +7517,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M137" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N137" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -8667,14 +7569,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M138" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N138" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -8727,14 +7621,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M139" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N139" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -8787,14 +7673,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M140" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N140" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -8847,14 +7725,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M141" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N141" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -8907,14 +7777,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M142" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N142" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -8967,14 +7829,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M143" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N143" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -9027,14 +7881,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M144" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N144" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -9087,14 +7933,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M145" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N145" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -9147,14 +7985,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M146" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N146" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -9190,7 +8020,7 @@
         <v>22031.6341269842</v>
       </c>
       <c r="I147" t="n">
-        <v>6385.980906372232</v>
+        <v>0</v>
       </c>
       <c r="J147" t="inlineStr">
         <is>
@@ -9206,14 +8036,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M147" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N147" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -9250,7 +8072,7 @@
         <v>22264.9020634921</v>
       </c>
       <c r="I148" t="n">
-        <v>6453.594801012203</v>
+        <v>0</v>
       </c>
       <c r="J148" t="inlineStr">
         <is>
@@ -9266,14 +8088,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M148" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N148" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -9328,14 +8142,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M149" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N149" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -9368,7 +8174,7 @@
         <v>22498.17</v>
       </c>
       <c r="I150" t="n">
-        <v>6521.208695652173</v>
+        <v>0</v>
       </c>
       <c r="J150" t="inlineStr">
         <is>
@@ -9384,14 +8190,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M150" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N150" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="151">
@@ -9424,7 +8222,7 @@
         <v>22614.803968254</v>
       </c>
       <c r="I151" t="n">
-        <v>6555.015642972174</v>
+        <v>0</v>
       </c>
       <c r="J151" t="inlineStr">
         <is>
@@ -9440,14 +8238,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M151" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N151" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="152">
@@ -9480,7 +8270,7 @@
         <v>22731.437936508</v>
       </c>
       <c r="I152" t="n">
-        <v>6588.822590292173</v>
+        <v>0</v>
       </c>
       <c r="J152" t="inlineStr">
         <is>
@@ -9496,14 +8286,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M152" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N152" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="153">
@@ -9536,7 +8318,7 @@
         <v>22848.0719047619</v>
       </c>
       <c r="I153" t="n">
-        <v>6622.629537612144</v>
+        <v>0</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
@@ -9552,14 +8334,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M153" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N153" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="154">
@@ -9598,7 +8372,7 @@
         <v>22964.7058730159</v>
       </c>
       <c r="I154" t="n">
-        <v>6656.436484932145</v>
+        <v>0</v>
       </c>
       <c r="J154" t="inlineStr">
         <is>
@@ -9614,14 +8388,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M154" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N154" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -9676,14 +8442,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M155" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N155" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -9720,7 +8478,7 @@
         <v>23197.9738095238</v>
       </c>
       <c r="I156" t="n">
-        <v>6724.050379572115</v>
+        <v>0</v>
       </c>
       <c r="J156" t="inlineStr">
         <is>
@@ -9736,14 +8494,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M156" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N156" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="157">
@@ -9780,7 +8530,7 @@
         <v>23314.6077777778</v>
       </c>
       <c r="I157" t="n">
-        <v>6757.857326892115</v>
+        <v>0</v>
       </c>
       <c r="J157" t="inlineStr">
         <is>
@@ -9796,14 +8546,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M157" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N157" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="158">
@@ -9840,7 +8582,7 @@
         <v>23431.2417460318</v>
       </c>
       <c r="I158" t="n">
-        <v>6791.664274212116</v>
+        <v>0</v>
       </c>
       <c r="J158" t="inlineStr">
         <is>
@@ -9856,14 +8598,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M158" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N158" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="159">
@@ -9917,14 +8651,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M159" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N159" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -9977,14 +8703,6 @@
           <t>PENDIENTE DE PAGO</t>
         </is>
       </c>
-      <c r="M160" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N160" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -10016,7 +8734,7 @@
         <v>2322049.968253971</v>
       </c>
       <c r="I161" t="n">
-        <v>1621505.91551645</v>
+        <v>0</v>
       </c>
       <c r="J161" t="inlineStr">
         <is>
@@ -10032,14 +8750,6 @@
         <is>
           <t>PENDIENTE DE PAGO</t>
         </is>
-      </c>
-      <c r="M161" t="inlineStr">
-        <is>
-          <t>2026-03-19T16:33:22.964043</t>
-        </is>
-      </c>
-      <c r="N161" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>